<commit_message>
modificaciones horarios y compras
</commit_message>
<xml_diff>
--- a/public/downloads/template_import_companies.xlsx
+++ b/public/downloads/template_import_companies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20368"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\laravel6_admin\public\downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\S&amp;I\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365ED636-B0DB-4C19-AC6F-2F2085350C10}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9427674-827F-464A-B68F-595FBB55A8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{1FF9B4F7-F8F4-4B01-9217-FACB22EB79B0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{1FF9B4F7-F8F4-4B01-9217-FACB22EB79B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>razon social</t>
   </si>
@@ -48,10 +48,19 @@
     <t>forma pago</t>
   </si>
   <si>
-    <t>dia pago</t>
-  </si>
-  <si>
     <t>poblacion</t>
+  </si>
+  <si>
+    <t>iban</t>
+  </si>
+  <si>
+    <t>condicion pago</t>
+  </si>
+  <si>
+    <t>cuenta gastos</t>
+  </si>
+  <si>
+    <t>concepto general</t>
   </si>
 </sst>
 </file>
@@ -403,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20B5E0C7-727B-4771-88C2-3D126F740539}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16.109375" customWidth="1"/>
@@ -411,7 +420,7 @@
     <col min="8" max="8" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -428,7 +437,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -437,7 +446,16 @@
         <v>6</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>